<commit_message>
Add ability to track and match specific product lots
Integrate 'Marka' (brand/lot) field into sales and purchase records, including API, UI, and data parsing updates, to enable more precise reconciliation and matching.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: e62cc95f-4e93-4f53-8634-82fafdea1c01
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: f8df9e80-9b9e-4c54-8421-7f91841ae7f1
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/33e7ad11-3f82-4d47-b09a-b6c5acdba6ca/e62cc95f-4e93-4f53-8634-82fafdea1c01/gYsgv8q
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/artifacts/reconciliation-app/public/purchase_template.xlsx
+++ b/artifacts/reconciliation-app/public/purchase_template.xlsx
@@ -397,19 +397,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:G4"/>
   <cols>
-    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
     <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="8.83203125" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" customWidth="1"/>
     <col min="5" max="5" width="8.83203125" customWidth="1"/>
-    <col min="6" max="6" width="10.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Date</v>
+        <v>Date / Bill Date</v>
       </c>
       <c r="B1" t="str">
         <v>Purchase Date</v>
@@ -418,78 +419,90 @@
         <v>Item</v>
       </c>
       <c r="D1" t="str">
-        <v>Qty</v>
+        <v>Qty (QTL)</v>
       </c>
       <c r="E1" t="str">
         <v>Rate</v>
       </c>
       <c r="F1" t="str">
         <v>Amount</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Marka</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>01-Apr-2026</v>
+        <v>20/04/2025</v>
       </c>
       <c r="B2" t="str">
-        <v>01-Apr-2026</v>
+        <v>15/04/2025</v>
       </c>
       <c r="C2" t="str">
-        <v>Wheat</v>
-      </c>
-      <c r="D2" t="str">
-        <v>100</v>
-      </c>
-      <c r="E2" t="str">
-        <v>2140</v>
-      </c>
-      <c r="F2" t="str">
-        <v>214000</v>
+        <v>Onion</v>
+      </c>
+      <c r="D2">
+        <v>120.5</v>
+      </c>
+      <c r="E2">
+        <v>850</v>
+      </c>
+      <c r="F2">
+        <v>102425</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Nashik Red</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>02-Apr-2026</v>
+        <v>21/04/2025</v>
       </c>
       <c r="B3" t="str">
-        <v>02-Apr-2026</v>
+        <v>16/04/2025</v>
       </c>
       <c r="C3" t="str">
-        <v>Soybean</v>
-      </c>
-      <c r="D3" t="str">
-        <v>50</v>
-      </c>
-      <c r="E3" t="str">
-        <v>4480</v>
-      </c>
-      <c r="F3" t="str">
-        <v>224000</v>
+        <v>Wheat</v>
+      </c>
+      <c r="D3">
+        <v>80</v>
+      </c>
+      <c r="E3">
+        <v>2150</v>
+      </c>
+      <c r="F3">
+        <v>172000</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Sharbati</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>03-Apr-2026</v>
+        <v>22/04/2025</v>
       </c>
       <c r="B4" t="str">
-        <v>03-Apr-2026</v>
+        <v>17/04/2025</v>
       </c>
       <c r="C4" t="str">
-        <v>Onion</v>
-      </c>
-      <c r="D4" t="str">
-        <v>80</v>
-      </c>
-      <c r="E4" t="str">
-        <v>1790</v>
-      </c>
-      <c r="F4" t="str">
-        <v>143200</v>
+        <v>Soybean</v>
+      </c>
+      <c r="D4">
+        <v>50</v>
+      </c>
+      <c r="E4">
+        <v>4500</v>
+      </c>
+      <c r="F4">
+        <v>225000</v>
+      </c>
+      <c r="G4" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>